<commit_message>
Sets CO2 budget to infinity
Modifies the CO2 budget to 'infinity' for the initial year of each time window. This change reflects a shift in the project's approach to carbon emissions constraints, allowing for unbounded CO2 emissions in the initial stages.
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0310EB8-B198-46BC-9B5F-FD6C789E7A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E034B45A-4AA2-4BBC-AA23-567A238680B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" tabRatio="796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="105">
   <si>
     <t>t</t>
   </si>
@@ -2951,8 +2951,8 @@
       <c r="A6" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="61">
-        <v>4426360000</v>
+      <c r="B6" s="61" t="s">
+        <v>27</v>
       </c>
       <c r="C6" s="29" t="s">
         <v>72</v>

</xml_diff>

<commit_message>
New Energy Mix for Start
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE1CACB3-5E98-40DC-AEBB-980362CE09E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A69FA6-F45F-4F81-AEC1-E8334110485A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="107">
   <si>
     <t>t</t>
   </si>
@@ -317,9 +317,6 @@
     <t>Coal Plant</t>
   </si>
   <si>
-    <t>Coal Lignite</t>
-  </si>
-  <si>
     <t>Gas Plant (CCGT)</t>
   </si>
   <si>
@@ -353,35 +350,43 @@
     <t>EU27.Gas plant</t>
   </si>
   <si>
-    <t>Coal CCUS</t>
-  </si>
-  <si>
-    <t>Coal Lignite CCUS</t>
-  </si>
-  <si>
     <t>Gas Plant (CCGT) CCUS</t>
   </si>
   <si>
-    <t>Piped Gas</t>
-  </si>
-  <si>
-    <t>Gas Plant (CCGT) LNG</t>
-  </si>
-  <si>
-    <t>LNG</t>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>Lignite Plant</t>
+  </si>
+  <si>
+    <t>Other non-res</t>
+  </si>
+  <si>
+    <t>Oil Plant</t>
+  </si>
+  <si>
+    <t>Coal Plant CCUS</t>
+  </si>
+  <si>
+    <t>Lignite Plant CCUS</t>
+  </si>
+  <si>
+    <t>Gas</t>
+  </si>
+  <si>
+    <t>Slack</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="45">
     <font>
@@ -692,7 +697,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="72">
+  <fills count="70">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1056,12 +1061,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1078,14 +1077,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="21">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -1314,15 +1307,6 @@
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1765,7 +1749,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1890,39 +1874,28 @@
     <xf numFmtId="0" fontId="0" fillId="24" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="66" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="67" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="68" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="67" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="67" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="68" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="0" fillId="69" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="0" fillId="68" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="70" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="69" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="66" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="71" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="66" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" indent="2"/>
-    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="437">
     <cellStyle name="20 % - Akzent1" xfId="233" builtinId="30" customBuiltin="1"/>
@@ -2363,7 +2336,7 @@
     <cellStyle name="Zelle überprüfen 4" xfId="214" xr:uid="{00000000-0005-0000-0000-000092010000}"/>
     <cellStyle name="Zelle überprüfen 5" xfId="215" xr:uid="{00000000-0005-0000-0000-000093010000}"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="47">
     <dxf>
       <border>
         <top style="thin">
@@ -2480,6 +2453,223 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -2920,7 +3110,7 @@
       <c r="A4" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="59" t="s">
         <v>27</v>
       </c>
       <c r="C4" s="29" t="s">
@@ -2942,7 +3132,7 @@
       <c r="A6" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="58" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="29" t="s">
@@ -2950,7 +3140,7 @@
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="B7" s="61"/>
+      <c r="B7" s="58"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2977,7 +3167,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2992,96 +3182,96 @@
       <c r="A3" s="5">
         <v>1</v>
       </c>
-      <c r="B3" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B3" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="5">
         <v>2</v>
       </c>
-      <c r="B4" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B4" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="5">
         <v>3</v>
       </c>
-      <c r="B5" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B5" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="5">
         <v>4</v>
       </c>
-      <c r="B6" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B6" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="5">
         <v>5</v>
       </c>
-      <c r="B7" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B7" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="5">
         <v>6</v>
       </c>
-      <c r="B8" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B8" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="5">
         <v>7</v>
       </c>
-      <c r="B9" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B9" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="5">
         <v>8</v>
       </c>
-      <c r="B10" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B10" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="5">
         <v>9</v>
       </c>
-      <c r="B11" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B11" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="5">
         <v>10</v>
       </c>
-      <c r="B12" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B12" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="5">
         <v>11</v>
       </c>
-      <c r="B13" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B13" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="5">
         <v>12</v>
       </c>
-      <c r="B14" s="60">
-        <v>0.20699999999999999</v>
+      <c r="B14" s="27">
+        <v>0.33750000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -3132,10 +3322,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>97</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -3167,7 +3357,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B2" s="7">
         <v>280000000</v>
@@ -3187,7 +3377,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="3" customWidth="1"/>
@@ -3221,7 +3411,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>1</v>
@@ -3244,7 +3434,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>35</v>
@@ -3267,7 +3457,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>36</v>
@@ -3287,10 +3477,10 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>5</v>
@@ -3298,8 +3488,8 @@
       <c r="D5">
         <v>22.68</v>
       </c>
-      <c r="E5" s="7">
-        <v>319200000</v>
+      <c r="E5" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>27</v>
@@ -3307,7 +3497,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>25</v>
@@ -3327,10 +3517,10 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>5</v>
@@ -3347,10 +3537,10 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>5</v>
@@ -3367,10 +3557,10 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>5</v>
@@ -3387,31 +3577,54 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D10">
-        <v>23.62</v>
+        <v>33.119999999999997</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>27</v>
       </c>
       <c r="F10" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11">
+        <v>33.119999999999997</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B1:F4" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
-  <conditionalFormatting sqref="B8:B10">
-    <cfRule type="expression" dxfId="22" priority="1">
+  <conditionalFormatting sqref="B8:B11">
+    <cfRule type="expression" dxfId="37" priority="10">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="36" priority="1"/>
   </conditionalFormatting>
   <dataValidations xWindow="307" yWindow="342" count="3">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Commodity price (€/MWh)" prompt="Cost for purchasing one unit (MWh) of a stock or buy commodity. Revenue for selling one unit (MWh) of a sell commodity. Cost for creating one unit of environmental commodity._x000a__x000a_Multiplier for sheet &quot;Buy-Sell-Price&quot; for commodity types &quot;Buy&quot; and &quot;Sell&quot;._x000a_" sqref="D1" xr:uid="{00000000-0002-0000-0200-000000000000}"/>
@@ -3428,7 +3641,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="3" customWidth="1"/>
@@ -3496,46 +3709,46 @@
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B2" s="49" t="s">
-        <v>84</v>
-      </c>
-      <c r="C2" s="50">
-        <v>46710</v>
+        <v>93</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="20">
+        <v>56122</v>
       </c>
       <c r="D2" s="20">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E2" s="20">
         <v>0</v>
       </c>
-      <c r="F2" s="51">
-        <v>46710</v>
-      </c>
-      <c r="G2" s="52" t="s">
+      <c r="F2" s="20">
+        <v>56122</v>
+      </c>
+      <c r="G2" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="53">
-        <v>0</v>
+      <c r="H2" s="51">
+        <v>0.5</v>
       </c>
       <c r="I2" s="54">
-        <v>2731780.3800000004</v>
-      </c>
-      <c r="J2" s="54">
-        <v>9923.6103600000006</v>
-      </c>
-      <c r="K2" s="54">
-        <v>0</v>
-      </c>
-      <c r="L2" s="55">
+        <v>1784013.3447999998</v>
+      </c>
+      <c r="J2" s="55">
+        <v>28544.213516800002</v>
+      </c>
+      <c r="K2" s="52">
+        <v>2.7</v>
+      </c>
+      <c r="L2" s="53">
         <v>0</v>
       </c>
       <c r="M2" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N2" s="55">
-        <v>60</v>
+      <c r="N2" s="53">
+        <v>40</v>
       </c>
       <c r="O2" s="28" t="e">
         <v>#N/A</v>
@@ -3543,46 +3756,46 @@
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B3" s="49" t="s">
-        <v>85</v>
-      </c>
-      <c r="C3" s="50">
-        <v>59840</v>
+        <v>93</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="20">
+        <v>43599</v>
       </c>
       <c r="D3" s="20">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E3" s="20">
         <v>0</v>
       </c>
-      <c r="F3" s="51">
-        <v>59840</v>
-      </c>
-      <c r="G3" s="52" t="s">
+      <c r="F3" s="20">
+        <v>43599</v>
+      </c>
+      <c r="G3" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H3" s="53">
-        <v>0</v>
-      </c>
-      <c r="I3" s="55">
-        <v>3345037.2</v>
-      </c>
-      <c r="J3" s="55">
-        <v>28432.799999999999</v>
-      </c>
-      <c r="K3" s="55">
-        <v>0.35699999999999998</v>
-      </c>
-      <c r="L3" s="55">
+      <c r="H3" s="51">
+        <v>0.65</v>
+      </c>
+      <c r="I3" s="52">
+        <v>2230016.6809999999</v>
+      </c>
+      <c r="J3" s="52">
+        <v>52182.390330800001</v>
+      </c>
+      <c r="K3" s="53">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="L3" s="53">
         <v>0</v>
       </c>
       <c r="M3" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N3" s="55">
-        <v>50</v>
+      <c r="N3" s="53">
+        <v>40</v>
       </c>
       <c r="O3" s="28" t="e">
         <v>#N/A</v>
@@ -3590,46 +3803,46 @@
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B4" s="49" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="50">
-        <v>53560</v>
+        <v>93</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="20">
+        <v>187303</v>
       </c>
       <c r="D4" s="20">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E4" s="20">
         <v>0</v>
       </c>
-      <c r="F4" s="50">
-        <v>53560</v>
-      </c>
-      <c r="G4" s="52" t="s">
+      <c r="F4" s="20">
+        <v>999999</v>
+      </c>
+      <c r="G4" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="53">
-        <v>0.5</v>
-      </c>
-      <c r="I4" s="56">
-        <v>1784013.3447999998</v>
-      </c>
-      <c r="J4" s="57">
-        <v>28544.213516800002</v>
-      </c>
-      <c r="K4" s="54">
-        <v>2.7</v>
-      </c>
-      <c r="L4" s="55">
+      <c r="H4" s="3">
+        <v>0</v>
+      </c>
+      <c r="I4" s="52">
+        <v>802808.92800000007</v>
+      </c>
+      <c r="J4" s="52">
+        <v>16725.186000000002</v>
+      </c>
+      <c r="K4" s="53">
+        <v>2.6</v>
+      </c>
+      <c r="L4" s="54">
         <v>0</v>
       </c>
       <c r="M4" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N4" s="55">
-        <v>40</v>
+      <c r="N4" s="53">
+        <v>25</v>
       </c>
       <c r="O4" s="28" t="e">
         <v>#N/A</v>
@@ -3637,46 +3850,46 @@
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B5" s="49" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" s="50">
-        <v>43590</v>
+        <v>93</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="20">
+        <v>13483</v>
       </c>
       <c r="D5" s="20">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E5" s="20">
         <v>0</v>
       </c>
-      <c r="F5" s="50">
-        <v>43590</v>
-      </c>
-      <c r="G5" s="52" t="s">
+      <c r="F5" s="20">
+        <v>13483</v>
+      </c>
+      <c r="G5" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="53">
-        <v>0.65</v>
-      </c>
-      <c r="I5" s="54">
-        <v>2230016.6809999999</v>
-      </c>
-      <c r="J5" s="54">
-        <v>52182.390330800001</v>
-      </c>
-      <c r="K5" s="55">
-        <v>4.5999999999999996</v>
-      </c>
-      <c r="L5" s="55">
+      <c r="H5" s="3">
+        <v>0</v>
+      </c>
+      <c r="I5" s="61">
+        <v>5648000</v>
+      </c>
+      <c r="J5" s="60">
+        <v>16725.186000000002</v>
+      </c>
+      <c r="K5" s="61">
+        <v>2.6</v>
+      </c>
+      <c r="L5" s="54">
         <v>0</v>
       </c>
       <c r="M5" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N5" s="55">
-        <v>40</v>
+      <c r="N5" s="53">
+        <v>25</v>
       </c>
       <c r="O5" s="28" t="e">
         <v>#N/A</v>
@@ -3684,45 +3897,45 @@
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="49" t="s">
-        <v>88</v>
-      </c>
-      <c r="C6" s="50">
-        <v>132230</v>
+        <v>93</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="20">
+        <v>14578</v>
       </c>
       <c r="D6" s="20">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E6" s="20">
         <v>0</v>
       </c>
-      <c r="F6" s="63">
-        <v>999999</v>
-      </c>
-      <c r="G6" s="52" t="s">
+      <c r="F6" s="20">
+        <v>14578</v>
+      </c>
+      <c r="G6" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="53">
-        <v>0</v>
-      </c>
-      <c r="I6" s="54">
-        <v>802808.92800000007</v>
-      </c>
-      <c r="J6" s="54">
+      <c r="H6" s="3">
+        <v>0</v>
+      </c>
+      <c r="I6" s="61">
+        <v>5648000</v>
+      </c>
+      <c r="J6" s="60">
         <v>16725.186000000002</v>
       </c>
-      <c r="K6" s="55">
+      <c r="K6" s="61">
         <v>2.6</v>
       </c>
-      <c r="L6" s="56">
+      <c r="L6" s="54">
         <v>0</v>
       </c>
       <c r="M6" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N6" s="55">
+      <c r="N6" s="53">
         <v>25</v>
       </c>
       <c r="O6" s="28" t="e">
@@ -3731,46 +3944,46 @@
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B7" s="49" t="s">
-        <v>89</v>
-      </c>
-      <c r="C7" s="50">
-        <v>94200</v>
+        <v>93</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="20">
+        <v>0</v>
       </c>
       <c r="D7" s="20">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E7" s="20">
         <v>0</v>
       </c>
-      <c r="F7" s="50">
-        <v>94200</v>
-      </c>
-      <c r="G7" s="52" t="s">
+      <c r="F7" s="20">
+        <v>100000</v>
+      </c>
+      <c r="G7" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="53">
-        <v>0</v>
-      </c>
-      <c r="I7" s="54">
-        <v>5909565.7200000007</v>
-      </c>
-      <c r="J7" s="57">
-        <v>133801.48800000001</v>
-      </c>
-      <c r="K7" s="54">
-        <v>7.1</v>
-      </c>
-      <c r="L7" s="55">
+      <c r="H7" s="51">
+        <v>0.5</v>
+      </c>
+      <c r="I7" s="53">
+        <v>3791028.3572399998</v>
+      </c>
+      <c r="J7" s="53">
+        <v>84183.129702000006</v>
+      </c>
+      <c r="K7" s="53">
+        <v>6.75</v>
+      </c>
+      <c r="L7" s="54">
         <v>0</v>
       </c>
       <c r="M7" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N7" s="55">
-        <v>60</v>
+      <c r="N7" s="53">
+        <v>40</v>
       </c>
       <c r="O7" s="28" t="e">
         <v>#N/A</v>
@@ -3778,46 +3991,46 @@
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B8" s="49" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="50">
-        <v>20420</v>
+        <v>93</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C8" s="20">
+        <v>0</v>
       </c>
       <c r="D8" s="20">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E8" s="20">
         <v>0</v>
       </c>
       <c r="F8" s="20">
-        <v>999999999999</v>
-      </c>
-      <c r="G8" s="52" t="s">
+        <v>100000</v>
+      </c>
+      <c r="G8" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="53">
-        <v>0</v>
-      </c>
-      <c r="I8" s="58">
-        <v>5648000</v>
-      </c>
-      <c r="J8" s="58">
-        <v>0</v>
-      </c>
-      <c r="K8" s="58">
-        <v>44.2</v>
-      </c>
-      <c r="L8" s="55">
+      <c r="H8" s="51">
+        <v>0.65</v>
+      </c>
+      <c r="I8" s="53">
+        <v>4014030.0248799999</v>
+      </c>
+      <c r="J8" s="53">
+        <v>76489.572146799997</v>
+      </c>
+      <c r="K8" s="53">
+        <v>6.96</v>
+      </c>
+      <c r="L8" s="54">
         <v>0</v>
       </c>
       <c r="M8" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N8" s="55">
-        <v>25</v>
+      <c r="N8" s="53">
+        <v>40</v>
       </c>
       <c r="O8" s="28" t="e">
         <v>#N/A</v>
@@ -3825,12 +4038,12 @@
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="49" t="s">
-        <v>99</v>
-      </c>
-      <c r="C9" s="50">
+        <v>93</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="20">
         <v>0</v>
       </c>
       <c r="D9" s="20">
@@ -3839,32 +4052,32 @@
       <c r="E9" s="20">
         <v>0</v>
       </c>
-      <c r="F9" s="50">
-        <v>0</v>
-      </c>
-      <c r="G9" s="52" t="s">
+      <c r="F9" s="20">
+        <v>100000</v>
+      </c>
+      <c r="G9" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="53">
-        <v>0.5</v>
-      </c>
-      <c r="I9" s="55">
-        <v>3791028.3572399998</v>
-      </c>
-      <c r="J9" s="55">
-        <v>84183.129702000006</v>
-      </c>
-      <c r="K9" s="55">
-        <v>6.75</v>
-      </c>
-      <c r="L9" s="56">
+      <c r="H9" s="3">
+        <v>0</v>
+      </c>
+      <c r="I9" s="53">
+        <v>1951271.6999999997</v>
+      </c>
+      <c r="J9" s="53">
+        <v>45715.5</v>
+      </c>
+      <c r="K9" s="53">
+        <v>3.46</v>
+      </c>
+      <c r="L9" s="54">
         <v>0</v>
       </c>
       <c r="M9" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N9" s="55">
-        <v>40</v>
+      <c r="N9" s="53">
+        <v>25</v>
       </c>
       <c r="O9" s="28" t="e">
         <v>#N/A</v>
@@ -3872,46 +4085,46 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="C10" s="50">
-        <v>0</v>
+        <v>88</v>
+      </c>
+      <c r="C10" s="20">
+        <v>94198</v>
       </c>
       <c r="D10" s="20">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="E10" s="20">
         <v>0</v>
       </c>
-      <c r="F10" s="50">
-        <v>0</v>
-      </c>
-      <c r="G10" s="52" t="s">
+      <c r="F10" s="20">
+        <v>94198</v>
+      </c>
+      <c r="G10" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="53">
-        <v>0.65</v>
-      </c>
-      <c r="I10" s="55">
-        <v>4014030.0248799999</v>
+      <c r="H10" s="3">
+        <v>0</v>
+      </c>
+      <c r="I10" s="52">
+        <v>5909565.7200000007</v>
       </c>
       <c r="J10" s="55">
-        <v>76489.572146799997</v>
-      </c>
-      <c r="K10" s="55">
-        <v>6.96</v>
-      </c>
-      <c r="L10" s="56">
+        <v>133801.48800000001</v>
+      </c>
+      <c r="K10" s="52">
+        <v>7.1</v>
+      </c>
+      <c r="L10" s="53">
         <v>0</v>
       </c>
       <c r="M10" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N10" s="55">
-        <v>40</v>
+      <c r="N10" s="53">
+        <v>60</v>
       </c>
       <c r="O10" s="28" t="e">
         <v>#N/A</v>
@@ -3919,46 +4132,46 @@
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>101</v>
-      </c>
-      <c r="C11" s="64">
-        <v>0</v>
+        <v>84</v>
+      </c>
+      <c r="C11" s="20">
+        <v>46703</v>
       </c>
       <c r="D11" s="20">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E11" s="20">
         <v>0</v>
       </c>
-      <c r="F11" s="50">
-        <v>0</v>
-      </c>
-      <c r="G11" s="52" t="s">
+      <c r="F11" s="20">
+        <v>46703</v>
+      </c>
+      <c r="G11" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H11" s="53">
-        <v>0</v>
-      </c>
-      <c r="I11" s="55">
-        <v>1951271.6999999997</v>
-      </c>
-      <c r="J11" s="55">
-        <v>45715.5</v>
-      </c>
-      <c r="K11" s="55">
-        <v>3.46</v>
-      </c>
-      <c r="L11" s="56">
+      <c r="H11" s="3">
+        <v>0</v>
+      </c>
+      <c r="I11" s="52">
+        <v>2731780.3800000004</v>
+      </c>
+      <c r="J11" s="52">
+        <v>9923.6103600000006</v>
+      </c>
+      <c r="K11" s="52">
+        <v>0</v>
+      </c>
+      <c r="L11" s="53">
         <v>0</v>
       </c>
       <c r="M11" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N11" s="55">
-        <v>25</v>
+      <c r="N11" s="53">
+        <v>60</v>
       </c>
       <c r="O11" s="28" t="e">
         <v>#N/A</v>
@@ -3966,96 +4179,178 @@
     </row>
     <row r="12" spans="1:15">
       <c r="A12" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B12" s="59" t="s">
-        <v>103</v>
-      </c>
-      <c r="C12" s="50">
-        <v>56670</v>
+        <v>93</v>
+      </c>
+      <c r="B12" s="49" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="20">
+        <v>61218</v>
       </c>
       <c r="D12" s="20">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E12" s="20">
         <v>0</v>
       </c>
-      <c r="F12" s="63">
-        <v>999999</v>
-      </c>
-      <c r="G12" s="52" t="s">
+      <c r="F12" s="20">
+        <v>61218</v>
+      </c>
+      <c r="G12" s="50" t="s">
         <v>27</v>
       </c>
-      <c r="H12" s="53">
-        <v>0.25</v>
-      </c>
-      <c r="I12" s="54">
-        <v>802808.92800000007</v>
-      </c>
-      <c r="J12" s="54">
-        <v>16725.186000000002</v>
-      </c>
-      <c r="K12" s="55">
-        <v>2.6</v>
-      </c>
-      <c r="L12" s="56">
+      <c r="H12" s="3">
+        <v>0</v>
+      </c>
+      <c r="I12" s="53">
+        <v>3345037.2</v>
+      </c>
+      <c r="J12" s="53">
+        <v>28432.799999999999</v>
+      </c>
+      <c r="K12" s="53">
+        <v>0.35699999999999998</v>
+      </c>
+      <c r="L12" s="53">
         <v>0</v>
       </c>
       <c r="M12" s="42">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="N12" s="55">
+      <c r="N12" s="53">
+        <v>50</v>
+      </c>
+      <c r="O12" s="28" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
+      <c r="A13" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" s="20">
+        <v>18651</v>
+      </c>
+      <c r="D13" s="20">
+        <v>10</v>
+      </c>
+      <c r="E13" s="20">
+        <v>0</v>
+      </c>
+      <c r="F13" s="20">
+        <v>999999</v>
+      </c>
+      <c r="G13" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0</v>
+      </c>
+      <c r="I13" s="56">
+        <v>5648000</v>
+      </c>
+      <c r="J13" s="56">
+        <v>0</v>
+      </c>
+      <c r="K13" s="56">
+        <v>44.2</v>
+      </c>
+      <c r="L13" s="53">
+        <v>0</v>
+      </c>
+      <c r="M13" s="42">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="N13" s="53">
         <v>25</v>
       </c>
-      <c r="O12" s="28" t="e">
+      <c r="O13" s="28" t="e">
         <v>#N/A</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
-  <conditionalFormatting sqref="A1:XFD4">
-    <cfRule type="expression" dxfId="21" priority="12">
+  <conditionalFormatting sqref="A1:XFD1 P9:XFD16 P2:XFD4">
+    <cfRule type="expression" dxfId="35" priority="39">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B3 A2:A12 D2:E12">
-    <cfRule type="expression" dxfId="20" priority="10">
+  <conditionalFormatting sqref="A16 A17:XFD1048576">
+    <cfRule type="expression" dxfId="34" priority="40">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:B12">
-    <cfRule type="expression" dxfId="19" priority="3">
+  <conditionalFormatting sqref="B2:F9 C10:F13 H9:H13 H4:H6">
+    <cfRule type="expression" dxfId="33" priority="14">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="18" priority="5">
+  <conditionalFormatting sqref="A2:A4">
+    <cfRule type="expression" dxfId="32" priority="13">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F8">
-    <cfRule type="expression" dxfId="17" priority="7">
+  <conditionalFormatting sqref="A2:A13">
+    <cfRule type="expression" dxfId="31" priority="12">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H6">
-    <cfRule type="expression" dxfId="16" priority="2">
+  <conditionalFormatting sqref="B10">
+    <cfRule type="expression" dxfId="30" priority="11">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H11">
-    <cfRule type="expression" dxfId="15" priority="1">
+  <conditionalFormatting sqref="B11:B12">
+    <cfRule type="expression" dxfId="29" priority="10">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:K2">
-    <cfRule type="expression" dxfId="14" priority="9">
+  <conditionalFormatting sqref="B11:B12">
+    <cfRule type="expression" dxfId="28" priority="9">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P9:XFD17 A17 A18:XFD1048576">
-    <cfRule type="expression" dxfId="13" priority="13">
+  <conditionalFormatting sqref="B13">
+    <cfRule type="expression" dxfId="27" priority="8">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G4 G12:G13">
+    <cfRule type="expression" dxfId="26" priority="7">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2">
+    <cfRule type="expression" dxfId="25" priority="6">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7">
+    <cfRule type="expression" dxfId="24" priority="5">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I11:O11">
+    <cfRule type="expression" dxfId="23" priority="4">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I11:K11">
+    <cfRule type="expression" dxfId="22" priority="3">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I12:O12">
+    <cfRule type="expression" dxfId="21" priority="2">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:O2">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4084,7 +4379,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16.33203125" style="3" bestFit="1" customWidth="1"/>
@@ -4113,8 +4408,8 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="59" t="s">
-        <v>87</v>
+      <c r="A2" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>36</v>
@@ -4130,8 +4425,8 @@
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="59" t="s">
-        <v>87</v>
+      <c r="A3" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>35</v>
@@ -4148,8 +4443,8 @@
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="59" t="s">
-        <v>87</v>
+      <c r="A4" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>25</v>
@@ -4165,11 +4460,11 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="59" t="s">
-        <v>88</v>
+      <c r="A5" s="57" t="s">
+        <v>87</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>39</v>
@@ -4183,8 +4478,8 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="59" t="s">
-        <v>88</v>
+      <c r="A6" s="57" t="s">
+        <v>87</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>35</v>
@@ -4201,8 +4496,8 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="59" t="s">
-        <v>88</v>
+      <c r="A7" s="57" t="s">
+        <v>87</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>25</v>
@@ -4219,11 +4514,11 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="59" t="s">
+      <c r="A8" s="57" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>39</v>
@@ -4237,8 +4532,8 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="59" t="s">
-        <v>90</v>
+      <c r="A9" s="57" t="s">
+        <v>89</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>35</v>
@@ -4255,8 +4550,8 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="59" t="s">
-        <v>90</v>
+      <c r="A10" s="57" t="s">
+        <v>89</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>25</v>
@@ -4273,11 +4568,11 @@
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="59" t="s">
-        <v>89</v>
+      <c r="A11" s="57" t="s">
+        <v>88</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>39</v>
@@ -4291,8 +4586,8 @@
       </c>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="59" t="s">
-        <v>89</v>
+      <c r="A12" s="57" t="s">
+        <v>88</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>35</v>
@@ -4309,11 +4604,11 @@
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="59" t="s">
+      <c r="A13" s="57" t="s">
         <v>86</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>39</v>
@@ -4326,7 +4621,7 @@
       </c>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="59" t="s">
+      <c r="A14" s="57" t="s">
         <v>86</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -4344,7 +4639,7 @@
       </c>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="59" t="s">
+      <c r="A15" s="57" t="s">
         <v>86</v>
       </c>
       <c r="B15" s="4" t="s">
@@ -4362,7 +4657,7 @@
       </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="59" t="s">
+      <c r="A16" s="57" t="s">
         <v>84</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -4380,7 +4675,7 @@
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="59" t="s">
+      <c r="A17" s="57" t="s">
         <v>84</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -4398,7 +4693,7 @@
       </c>
     </row>
     <row r="18" spans="1:5">
-      <c r="A18" s="59" t="s">
+      <c r="A18" s="57" t="s">
         <v>85</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -4416,7 +4711,7 @@
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="59" t="s">
+      <c r="A19" s="57" t="s">
         <v>85</v>
       </c>
       <c r="B19" s="4" t="s">
@@ -4434,11 +4729,11 @@
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="59" t="s">
-        <v>99</v>
+      <c r="A20" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>39</v>
@@ -4452,8 +4747,8 @@
       </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="59" t="s">
-        <v>99</v>
+      <c r="A21" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>35</v>
@@ -4461,7 +4756,7 @@
       <c r="C21" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="65">
+      <c r="D21" s="24">
         <v>0.36</v>
       </c>
       <c r="E21" s="24" t="e">
@@ -4470,8 +4765,8 @@
       </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="59" t="s">
-        <v>99</v>
+      <c r="A22" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>25</v>
@@ -4479,7 +4774,7 @@
       <c r="C22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D22" s="66">
+      <c r="D22" s="24">
         <v>3.4180000000000002E-2</v>
       </c>
       <c r="E22" s="24" t="e">
@@ -4488,11 +4783,11 @@
       </c>
     </row>
     <row r="23" spans="1:5">
-      <c r="A23" s="59" t="s">
-        <v>100</v>
+      <c r="A23" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>39</v>
@@ -4506,8 +4801,8 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="59" t="s">
-        <v>100</v>
+      <c r="A24" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>35</v>
@@ -4515,7 +4810,7 @@
       <c r="C24" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="65">
+      <c r="D24" s="24">
         <v>0.32</v>
       </c>
       <c r="E24" s="24" t="e">
@@ -4524,8 +4819,8 @@
       </c>
     </row>
     <row r="25" spans="1:5">
-      <c r="A25" s="59" t="s">
-        <v>100</v>
+      <c r="A25" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>25</v>
@@ -4533,7 +4828,7 @@
       <c r="C25" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D25" s="66">
+      <c r="D25" s="24">
         <v>3.6299999999999999E-2</v>
       </c>
       <c r="E25" s="24" t="e">
@@ -4542,11 +4837,11 @@
       </c>
     </row>
     <row r="26" spans="1:5">
-      <c r="A26" s="59" t="s">
-        <v>101</v>
+      <c r="A26" s="57" t="s">
+        <v>98</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>39</v>
@@ -4560,8 +4855,8 @@
       </c>
     </row>
     <row r="27" spans="1:5">
-      <c r="A27" s="59" t="s">
-        <v>101</v>
+      <c r="A27" s="57" t="s">
+        <v>98</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>35</v>
@@ -4569,7 +4864,7 @@
       <c r="C27" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D27" s="65">
+      <c r="D27" s="24">
         <v>0.4</v>
       </c>
       <c r="E27" s="24" t="e">
@@ -4578,8 +4873,8 @@
       </c>
     </row>
     <row r="28" spans="1:5">
-      <c r="A28" s="59" t="s">
-        <v>101</v>
+      <c r="A28" s="57" t="s">
+        <v>98</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>25</v>
@@ -4587,7 +4882,7 @@
       <c r="C28" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D28" s="66">
+      <c r="D28" s="24">
         <v>2.0500000000000001E-2</v>
       </c>
       <c r="E28" s="24" t="e">
@@ -4596,11 +4891,11 @@
       </c>
     </row>
     <row r="29" spans="1:5">
-      <c r="A29" s="59" t="s">
-        <v>103</v>
+      <c r="A29" s="3" t="s">
+        <v>101</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>39</v>
@@ -4614,8 +4909,8 @@
       </c>
     </row>
     <row r="30" spans="1:5">
-      <c r="A30" s="59" t="s">
-        <v>103</v>
+      <c r="A30" s="3" t="s">
+        <v>101</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>35</v>
@@ -4624,7 +4919,7 @@
         <v>40</v>
       </c>
       <c r="D30" s="24">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="E30" s="24" t="e">
         <f>NA()</f>
@@ -4632,8 +4927,8 @@
       </c>
     </row>
     <row r="31" spans="1:5">
-      <c r="A31" s="59" t="s">
-        <v>103</v>
+      <c r="A31" s="3" t="s">
+        <v>101</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>25</v>
@@ -4642,37 +4937,91 @@
         <v>40</v>
       </c>
       <c r="D31" s="24">
-        <v>0.20499999999999999</v>
+        <v>0.26700000000000002</v>
       </c>
       <c r="E31" s="24" t="e">
-        <f>D31*E29</f>
+        <f>NA()</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" s="24">
+        <v>1</v>
+      </c>
+      <c r="E32" s="24" t="e">
+        <f>D32*E30</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="24">
+        <v>0.4</v>
+      </c>
+      <c r="E33" s="24" t="e">
+        <f>NA()</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D34" s="24">
+        <v>0.26700000000000002</v>
+      </c>
+      <c r="E34" s="24" t="e">
+        <f>NA()</f>
         <v>#N/A</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
-  <conditionalFormatting sqref="A1:XFD2 D2:D19 A3:C4 E3:XFD4 A5 A6:C7 E6:XFD7 A8:XFD12 A13:C15 E13:XFD15 A16:XFD19 A30:C31 E30:XFD31 A32:XFD1048576">
-    <cfRule type="expression" dxfId="12" priority="39">
+  <conditionalFormatting sqref="A1:XFD1 D2:D19 B3:C4 E3:XFD4 A5 A6:C7 E6:XFD7 A8:XFD12 A13:C15 E13:XFD15 A16:XFD19 A35:XFD1048576 B2:XFD2 F29:XFD34">
+    <cfRule type="expression" dxfId="19" priority="66">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B21:C25 C26:D26 B27:C27">
-    <cfRule type="expression" dxfId="11" priority="25">
+  <conditionalFormatting sqref="B21:C25 C26 B27:C27">
+    <cfRule type="expression" dxfId="18" priority="52">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20:E20 A20:A29 D23:E23">
-    <cfRule type="expression" dxfId="10" priority="26">
+  <conditionalFormatting sqref="B20:C20 A26:A28 E23 E20">
+    <cfRule type="expression" dxfId="17" priority="53">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:XFD5">
-    <cfRule type="expression" dxfId="9" priority="4">
+    <cfRule type="expression" dxfId="16" priority="31">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D7">
-    <cfRule type="dataBar" priority="36">
+  <conditionalFormatting sqref="D6:D7 D35:E1048576">
+    <cfRule type="dataBar" priority="63">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4686,7 +5035,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D8:D10 D5 E3:E4 E6:E7">
-    <cfRule type="dataBar" priority="45">
+    <cfRule type="dataBar" priority="72">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4699,8 +5048,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D13 D15">
-    <cfRule type="dataBar" priority="34">
+  <conditionalFormatting sqref="D15 D13">
+    <cfRule type="dataBar" priority="61">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4714,7 +5063,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15">
-    <cfRule type="dataBar" priority="32">
+    <cfRule type="dataBar" priority="59">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4727,165 +5076,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D20">
-    <cfRule type="dataBar" priority="28">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DF85B3E7-6D24-4702-AB47-0D47F71538F8}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D22">
-    <cfRule type="dataBar" priority="17">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F7E4DC53-D7B5-4205-8087-340EC79B984A}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="18">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-    <cfRule type="dataBar" priority="19">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BD4EE866-58E4-4CE7-814D-6232EE42462C}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D23">
-    <cfRule type="dataBar" priority="27">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{638DB081-4439-4940-9AE3-880EB91DD8D4}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D25">
-    <cfRule type="dataBar" priority="14">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4FA8C8CC-9E06-4AAF-9D36-B69E2717DF17}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="15">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-    <cfRule type="dataBar" priority="16">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{65B46255-DD72-4D46-B680-EA22FDABDF35}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D28">
-    <cfRule type="dataBar" priority="11">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6B773CE8-FE95-4E79-8BA2-717E6DDC4252}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-    <cfRule type="dataBar" priority="13">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B2637DB6-30FE-4484-B8A4-D99048727AA5}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D29">
-    <cfRule type="dataBar" priority="9">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{05321CB7-284A-4FA6-BF65-78097A8972CB}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D29:D31">
-    <cfRule type="expression" dxfId="6" priority="7">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-    <cfRule type="dataBar" priority="10">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{28824AAA-F1F2-4A7D-928D-3858A69D3F02}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D30:D31">
-    <cfRule type="dataBar" priority="8">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{565012B0-F520-423C-81F4-0556E4C75B40}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D2:E2 D2:D19">
-    <cfRule type="dataBar" priority="38">
+    <cfRule type="dataBar" priority="65">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4899,7 +5091,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11:E12">
-    <cfRule type="dataBar" priority="47">
+    <cfRule type="dataBar" priority="74">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4913,7 +5105,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D16:E17">
-    <cfRule type="dataBar" priority="41">
+    <cfRule type="dataBar" priority="68">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4927,7 +5119,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18:E19">
-    <cfRule type="dataBar" priority="40">
+    <cfRule type="dataBar" priority="67">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4940,8 +5132,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D32:E1048576 D1:E1">
-    <cfRule type="dataBar" priority="66">
+  <conditionalFormatting sqref="D1:E1">
+    <cfRule type="dataBar" priority="93">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4955,7 +5147,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5">
-    <cfRule type="dataBar" priority="5">
+    <cfRule type="dataBar" priority="32">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4969,7 +5161,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E8:E10">
-    <cfRule type="dataBar" priority="44">
+    <cfRule type="dataBar" priority="71">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4983,7 +5175,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E13:E15">
-    <cfRule type="dataBar" priority="42">
+    <cfRule type="dataBar" priority="69">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4997,7 +5189,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E20:E22">
-    <cfRule type="dataBar" priority="31">
+    <cfRule type="dataBar" priority="58">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5011,12 +5203,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E21:E22">
-    <cfRule type="expression" dxfId="5" priority="24">
+    <cfRule type="expression" dxfId="15" priority="51">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E23:E24">
-    <cfRule type="dataBar" priority="30">
+    <cfRule type="dataBar" priority="57">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5029,13 +5221,13 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E24:E29">
-    <cfRule type="expression" dxfId="4" priority="1">
+  <conditionalFormatting sqref="E24:E34">
+    <cfRule type="expression" dxfId="14" priority="28">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E25:E26">
-    <cfRule type="dataBar" priority="23">
+    <cfRule type="dataBar" priority="50">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5048,8 +5240,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E27 D26">
-    <cfRule type="dataBar" priority="29">
+  <conditionalFormatting sqref="E27">
+    <cfRule type="dataBar" priority="56">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5063,7 +5255,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E28">
-    <cfRule type="dataBar" priority="21">
+    <cfRule type="dataBar" priority="48">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5076,8 +5268,33 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F20:XFD28 B28:C28">
+    <cfRule type="expression" dxfId="13" priority="33">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:A4">
+    <cfRule type="expression" dxfId="12" priority="22">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A29:A31">
+    <cfRule type="expression" dxfId="11" priority="21">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A32:A34">
+    <cfRule type="expression" dxfId="10" priority="20">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C29 B30:C30">
+    <cfRule type="expression" dxfId="9" priority="18">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E29">
-    <cfRule type="dataBar" priority="2">
+    <cfRule type="dataBar" priority="17">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5085,12 +5302,126 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2C9C93EA-BC71-4CDD-B218-F0139631B6A8}</x14:id>
+          <x14:id>{300C6859-9C43-4AEC-AFC7-5EFBEDA5FFC9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E30:E31">
+  <conditionalFormatting sqref="E30">
+    <cfRule type="dataBar" priority="19">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{4F0D40E6-4588-4F1B-B566-71161E555644}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E31">
+    <cfRule type="dataBar" priority="16">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F85D4A2E-7508-48E4-B231-7EC9DFE30A3A}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31:C31">
+    <cfRule type="expression" dxfId="8" priority="13">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C32 B33:C33">
+    <cfRule type="expression" dxfId="7" priority="11">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E32">
+    <cfRule type="dataBar" priority="10">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{631841D2-B288-4E38-89D8-A83C71A694E2}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E33">
+    <cfRule type="dataBar" priority="12">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{11D952EA-6F71-484F-992F-FC230678E023}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E34">
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{66ACFE75-5158-4AB2-B574-39A4A5AFA58F}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B34:C34">
+    <cfRule type="expression" dxfId="6" priority="6">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20:A22">
+    <cfRule type="expression" dxfId="5" priority="5">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A23:A25">
+    <cfRule type="expression" dxfId="4" priority="4">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20:D34">
+    <cfRule type="expression" dxfId="3" priority="2">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20:D34">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{7AB2700A-6B81-40CE-9D8E-09F24EE45515}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20:D34">
     <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5099,14 +5430,9 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E4A87931-967F-4664-A132-1A1346D2C7A5}</x14:id>
+          <x14:id>{2A85A53E-8626-4C70-ACB0-05A059847601}</x14:id>
         </ext>
       </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F20:XFD29 B28:D29">
-    <cfRule type="expression" dxfId="3" priority="6">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -5131,7 +5457,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D6:D7</xm:sqref>
+          <xm:sqref>D6:D7 D35:E1048576</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{4EFF1923-5632-46D2-BEE4-19792B834F3E}">
@@ -5161,7 +5487,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D13 D15</xm:sqref>
+          <xm:sqref>D15 D13</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C12684E9-C44A-443A-881A-7ED428CB9718}">
@@ -5177,162 +5503,6 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>D15</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DF85B3E7-6D24-4702-AB47-0D47F71538F8}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D20</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F7E4DC53-D7B5-4205-8087-340EC79B984A}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <x14:cfRule type="dataBar" id="{BD4EE866-58E4-4CE7-814D-6232EE42462C}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D22</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{638DB081-4439-4940-9AE3-880EB91DD8D4}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D23</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4FA8C8CC-9E06-4AAF-9D36-B69E2717DF17}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <x14:cfRule type="dataBar" id="{65B46255-DD72-4D46-B680-EA22FDABDF35}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D25</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6B773CE8-FE95-4E79-8BA2-717E6DDC4252}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <x14:cfRule type="dataBar" id="{B2637DB6-30FE-4484-B8A4-D99048727AA5}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D28</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{05321CB7-284A-4FA6-BF65-78097A8972CB}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D29</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{28824AAA-F1F2-4A7D-928D-3858A69D3F02}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D29:D31</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{565012B0-F520-423C-81F4-0556E4C75B40}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D30:D31</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{E75D5CC6-8EBE-4E5D-B4DA-5515E5E7F357}">
@@ -5407,7 +5577,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D32:E1048576 D1:E1</xm:sqref>
+          <xm:sqref>D1:E1</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{3721D2A3-FECF-4A8D-8467-880D87B6D2BC}">
@@ -5512,7 +5682,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E27 D26</xm:sqref>
+          <xm:sqref>E27</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{A7C290DA-E617-4412-A5C5-3335857A068B}">
@@ -5530,7 +5700,7 @@
           <xm:sqref>E28</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2C9C93EA-BC71-4CDD-B218-F0139631B6A8}">
+          <x14:cfRule type="dataBar" id="{300C6859-9C43-4AEC-AFC7-5EFBEDA5FFC9}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5545,7 +5715,7 @@
           <xm:sqref>E29</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E4A87931-967F-4664-A132-1A1346D2C7A5}">
+          <x14:cfRule type="dataBar" id="{4F0D40E6-4588-4F1B-B566-71161E555644}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5557,7 +5727,97 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E30:E31</xm:sqref>
+          <xm:sqref>E30</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F85D4A2E-7508-48E4-B231-7EC9DFE30A3A}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E31</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{631841D2-B288-4E38-89D8-A83C71A694E2}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E32</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{11D952EA-6F71-484F-992F-FC230678E023}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E33</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{66ACFE75-5158-4AB2-B574-39A4A5AFA58F}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E34</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{7AB2700A-6B81-40CE-9D8E-09F24EE45515}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D20:D34</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{2A85A53E-8626-4C70-ACB0-05A059847601}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D20:D34</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -5769,7 +6029,7 @@
     </row>
     <row r="2" spans="1:23">
       <c r="A2" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B2" s="41" t="s">
         <v>81</v>
@@ -5838,7 +6098,7 @@
     </row>
     <row r="3" spans="1:23">
       <c r="A3" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B3" s="41" t="s">
         <v>82</v>
@@ -5908,7 +6168,7 @@
     </row>
     <row r="4" spans="1:23">
       <c r="A4" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" s="47" t="s">
         <v>83</v>
@@ -6108,7 +6368,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:2">

</xml_diff>

<commit_message>
Integrated the thermal efficiency into fuel and co2 emissions so elec is scaled to 1
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97A69FA6-F45F-4F81-AEC1-E8334110485A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1DD5CA-3F8A-48D5-A956-A4AC9E3200EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -1749,7 +1749,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1894,8 +1894,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="437">
     <cellStyle name="20 % - Akzent1" xfId="233" builtinId="30" customBuiltin="1"/>
@@ -2336,97 +2335,7 @@
     <cellStyle name="Zelle überprüfen 4" xfId="214" xr:uid="{00000000-0005-0000-0000-000092010000}"/>
     <cellStyle name="Zelle überprüfen 5" xfId="215" xr:uid="{00000000-0005-0000-0000-000093010000}"/>
   </cellStyles>
-  <dxfs count="47">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="27">
     <dxf>
       <border>
         <top style="thin">
@@ -2670,96 +2579,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3618,13 +3437,13 @@
   </sheetData>
   <autoFilter ref="B1:F4" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="26" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B8:B11">
-    <cfRule type="expression" dxfId="37" priority="10">
+    <cfRule type="expression" dxfId="25" priority="10">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="36" priority="1"/>
   </conditionalFormatting>
   <dataValidations xWindow="307" yWindow="342" count="3">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Commodity price (€/MWh)" prompt="Cost for purchasing one unit (MWh) of a stock or buy commodity. Revenue for selling one unit (MWh) of a sell commodity. Cost for creating one unit of environmental commodity._x000a__x000a_Multiplier for sheet &quot;Buy-Sell-Price&quot; for commodity types &quot;Buy&quot; and &quot;Sell&quot;._x000a_" sqref="D1" xr:uid="{00000000-0002-0000-0200-000000000000}"/>
@@ -3812,7 +3631,7 @@
         <v>187303</v>
       </c>
       <c r="D4" s="20">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E4" s="20">
         <v>0</v>
@@ -3824,7 +3643,7 @@
         <v>27</v>
       </c>
       <c r="H4" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I4" s="52">
         <v>802808.92800000007</v>
@@ -3873,13 +3692,13 @@
       <c r="H5" s="3">
         <v>0</v>
       </c>
-      <c r="I5" s="61">
+      <c r="I5">
         <v>5648000</v>
       </c>
       <c r="J5" s="60">
         <v>16725.186000000002</v>
       </c>
-      <c r="K5" s="61">
+      <c r="K5">
         <v>2.6</v>
       </c>
       <c r="L5" s="54">
@@ -3918,15 +3737,15 @@
         <v>27</v>
       </c>
       <c r="H6" s="3">
-        <v>0</v>
-      </c>
-      <c r="I6" s="61">
+        <v>0.1</v>
+      </c>
+      <c r="I6">
         <v>5648000</v>
       </c>
       <c r="J6" s="60">
         <v>16725.186000000002</v>
       </c>
-      <c r="K6" s="61">
+      <c r="K6">
         <v>2.6</v>
       </c>
       <c r="L6" s="54">
@@ -4059,7 +3878,7 @@
         <v>27</v>
       </c>
       <c r="H9" s="3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I9" s="53">
         <v>1951271.6999999997</v>
@@ -4106,7 +3925,7 @@
         <v>27</v>
       </c>
       <c r="H10" s="3">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I10" s="52">
         <v>5909565.7200000007</v>
@@ -4153,7 +3972,7 @@
         <v>27</v>
       </c>
       <c r="H11" s="3">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I11" s="52">
         <v>2731780.3800000004</v>
@@ -4200,7 +4019,7 @@
         <v>27</v>
       </c>
       <c r="H12" s="3">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="I12" s="53">
         <v>3345037.2</v>
@@ -4247,7 +4066,7 @@
         <v>27</v>
       </c>
       <c r="H13" s="3">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I13" s="56">
         <v>5648000</v>
@@ -4274,83 +4093,48 @@
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
-  <conditionalFormatting sqref="A1:XFD1 P9:XFD16 P2:XFD4">
-    <cfRule type="expression" dxfId="35" priority="39">
+  <conditionalFormatting sqref="A16 A17:XFD1048576">
+    <cfRule type="expression" dxfId="24" priority="41">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A16 A17:XFD1048576">
-    <cfRule type="expression" dxfId="34" priority="40">
+  <conditionalFormatting sqref="A2:F13">
+    <cfRule type="expression" dxfId="23" priority="9">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:F9 C10:F13 H9:H13 H4:H6">
-    <cfRule type="expression" dxfId="33" priority="14">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A4">
-    <cfRule type="expression" dxfId="32" priority="13">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A13">
-    <cfRule type="expression" dxfId="31" priority="12">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B10">
-    <cfRule type="expression" dxfId="30" priority="11">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11:B12">
-    <cfRule type="expression" dxfId="29" priority="10">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B11:B12">
-    <cfRule type="expression" dxfId="28" priority="9">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13">
-    <cfRule type="expression" dxfId="27" priority="8">
+  <conditionalFormatting sqref="A1:XFD1 P2:XFD4 P9:XFD16">
+    <cfRule type="expression" dxfId="22" priority="40">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G4 G12:G13">
-    <cfRule type="expression" dxfId="26" priority="7">
+    <cfRule type="expression" dxfId="21" priority="8">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2">
-    <cfRule type="expression" dxfId="25" priority="6">
+  <conditionalFormatting sqref="H4:H7">
+    <cfRule type="expression" dxfId="20" priority="6">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7">
-    <cfRule type="expression" dxfId="24" priority="5">
+  <conditionalFormatting sqref="H9:H13">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I11:O11">
-    <cfRule type="expression" dxfId="23" priority="4">
+  <conditionalFormatting sqref="H2:O2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I11:K11">
-    <cfRule type="expression" dxfId="22" priority="3">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I12:O12">
-    <cfRule type="expression" dxfId="21" priority="2">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I2:O2">
-    <cfRule type="expression" dxfId="20" priority="1">
+  <conditionalFormatting sqref="I11:O12">
+    <cfRule type="expression" dxfId="16" priority="3">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4418,10 +4202,10 @@
         <v>39</v>
       </c>
       <c r="D2" s="24">
-        <v>1</v>
+        <v>2.4390243902439024</v>
       </c>
       <c r="E2" s="24">
-        <v>2</v>
+        <v>2.4390243902439024</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -4435,11 +4219,10 @@
         <v>40</v>
       </c>
       <c r="D3" s="24">
-        <v>0.41</v>
-      </c>
-      <c r="E3" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E3" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -4453,10 +4236,10 @@
         <v>40</v>
       </c>
       <c r="D4" s="24">
-        <v>0.36299999999999999</v>
+        <v>0.88536585365853659</v>
       </c>
       <c r="E4" s="24">
-        <v>0.8</v>
+        <v>0.88536585365853659</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -4470,11 +4253,10 @@
         <v>39</v>
       </c>
       <c r="D5" s="24">
-        <v>1</v>
-      </c>
-      <c r="E5" s="24" t="e">
-        <f>D5*E3</f>
-        <v>#N/A</v>
+        <v>1.6666666666666667</v>
+      </c>
+      <c r="E5" s="24">
+        <v>1.6666666666666667</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4488,11 +4270,10 @@
         <v>40</v>
       </c>
       <c r="D6" s="24">
-        <v>0.6</v>
-      </c>
-      <c r="E6" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E6" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -4506,11 +4287,10 @@
         <v>40</v>
       </c>
       <c r="D7" s="24">
-        <v>0.20499999999999999</v>
-      </c>
-      <c r="E7" s="24" t="e">
-        <f>D7*E5</f>
-        <v>#N/A</v>
+        <v>0.34166666666666667</v>
+      </c>
+      <c r="E7" s="24">
+        <v>0.34166666666666667</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4524,11 +4304,10 @@
         <v>39</v>
       </c>
       <c r="D8" s="24">
-        <v>1</v>
-      </c>
-      <c r="E8" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>2.8571428571428572</v>
+      </c>
+      <c r="E8" s="24">
+        <v>2.8571428571428572</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -4542,11 +4321,10 @@
         <v>40</v>
       </c>
       <c r="D9" s="24">
-        <v>0.35</v>
-      </c>
-      <c r="E9" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E9" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -4562,9 +4340,8 @@
       <c r="D10" s="24">
         <v>0</v>
       </c>
-      <c r="E10" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+      <c r="E10" s="24">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -4578,11 +4355,10 @@
         <v>39</v>
       </c>
       <c r="D11" s="24">
-        <v>1</v>
-      </c>
-      <c r="E11" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>2.6315789473684212</v>
+      </c>
+      <c r="E11" s="24">
+        <v>2.6315789473684212</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -4596,11 +4372,10 @@
         <v>40</v>
       </c>
       <c r="D12" s="24">
-        <v>0.38</v>
-      </c>
-      <c r="E12" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E12" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -4614,10 +4389,10 @@
         <v>39</v>
       </c>
       <c r="D13" s="24">
-        <v>1</v>
+        <v>2.2222222222222223</v>
       </c>
       <c r="E13" s="24">
-        <v>1.4</v>
+        <v>2.2222222222222223</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -4631,11 +4406,10 @@
         <v>40</v>
       </c>
       <c r="D14" s="24">
-        <v>0.45</v>
-      </c>
-      <c r="E14" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E14" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -4649,11 +4423,10 @@
         <v>40</v>
       </c>
       <c r="D15" s="24">
-        <v>0.34179999999999999</v>
+        <v>0.75955555555555554</v>
       </c>
       <c r="E15" s="24">
-        <f>D15*E13</f>
-        <v>0.47851999999999995</v>
+        <v>0.75955555555555554</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -4669,9 +4442,8 @@
       <c r="D16" s="24">
         <v>1</v>
       </c>
-      <c r="E16" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+      <c r="E16" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -4687,9 +4459,8 @@
       <c r="D17" s="24">
         <v>1</v>
       </c>
-      <c r="E17" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+      <c r="E17" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -4705,9 +4476,8 @@
       <c r="D18" s="24">
         <v>1</v>
       </c>
-      <c r="E18" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+      <c r="E18" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -4723,9 +4493,8 @@
       <c r="D19" s="24">
         <v>1</v>
       </c>
-      <c r="E19" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+      <c r="E19" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -4739,11 +4508,10 @@
         <v>39</v>
       </c>
       <c r="D20" s="24">
-        <v>1</v>
-      </c>
-      <c r="E20" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>2.7777777777777777</v>
+      </c>
+      <c r="E20" s="24">
+        <v>2.7777777777777777</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -4757,11 +4525,10 @@
         <v>40</v>
       </c>
       <c r="D21" s="24">
-        <v>0.36</v>
-      </c>
-      <c r="E21" s="24" t="e">
-        <f>D21*E19</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E21" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -4775,11 +4542,10 @@
         <v>40</v>
       </c>
       <c r="D22" s="24">
-        <v>3.4180000000000002E-2</v>
-      </c>
-      <c r="E22" s="24" t="e">
-        <f>D22*E20</f>
-        <v>#N/A</v>
+        <v>9.4944444444444442E-2</v>
+      </c>
+      <c r="E22" s="24">
+        <v>9.4944444444444442E-2</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -4793,11 +4559,10 @@
         <v>39</v>
       </c>
       <c r="D23" s="24">
-        <v>1</v>
-      </c>
-      <c r="E23" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>3.125</v>
+      </c>
+      <c r="E23" s="24">
+        <v>3.125</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -4811,11 +4576,10 @@
         <v>40</v>
       </c>
       <c r="D24" s="24">
-        <v>0.32</v>
-      </c>
-      <c r="E24" s="24" t="e">
-        <f>D24*E21</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E24" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -4829,11 +4593,10 @@
         <v>40</v>
       </c>
       <c r="D25" s="24">
-        <v>3.6299999999999999E-2</v>
-      </c>
-      <c r="E25" s="24" t="e">
-        <f>D25*E23</f>
-        <v>#N/A</v>
+        <v>0.1134375</v>
+      </c>
+      <c r="E25" s="24">
+        <v>0.1134375</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -4847,11 +4610,10 @@
         <v>39</v>
       </c>
       <c r="D26" s="24">
-        <v>1</v>
-      </c>
-      <c r="E26" s="24" t="e">
-        <f>D26*E24</f>
-        <v>#N/A</v>
+        <v>2.5</v>
+      </c>
+      <c r="E26" s="24">
+        <v>2.5</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -4865,11 +4627,10 @@
         <v>40</v>
       </c>
       <c r="D27" s="24">
-        <v>0.4</v>
-      </c>
-      <c r="E27" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E27" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -4883,11 +4644,10 @@
         <v>40</v>
       </c>
       <c r="D28" s="24">
-        <v>2.0500000000000001E-2</v>
-      </c>
-      <c r="E28" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>5.1250000000000004E-2</v>
+      </c>
+      <c r="E28" s="24">
+        <v>5.1250000000000004E-2</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -4901,11 +4661,10 @@
         <v>39</v>
       </c>
       <c r="D29" s="24">
-        <v>1</v>
-      </c>
-      <c r="E29" s="24" t="e">
-        <f>D29*E27</f>
-        <v>#N/A</v>
+        <v>2.5</v>
+      </c>
+      <c r="E29" s="24">
+        <v>2.5</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -4919,11 +4678,10 @@
         <v>40</v>
       </c>
       <c r="D30" s="24">
-        <v>0.4</v>
-      </c>
-      <c r="E30" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E30" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -4937,11 +4695,10 @@
         <v>40</v>
       </c>
       <c r="D31" s="24">
-        <v>0.26700000000000002</v>
-      </c>
-      <c r="E31" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>0.66749999999999998</v>
+      </c>
+      <c r="E31" s="24">
+        <v>0.66749999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -4955,11 +4712,10 @@
         <v>39</v>
       </c>
       <c r="D32" s="24">
-        <v>1</v>
-      </c>
-      <c r="E32" s="24" t="e">
-        <f>D32*E30</f>
-        <v>#N/A</v>
+        <v>2.5</v>
+      </c>
+      <c r="E32" s="24">
+        <v>2.5</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -4973,11 +4729,10 @@
         <v>40</v>
       </c>
       <c r="D33" s="24">
-        <v>0.4</v>
-      </c>
-      <c r="E33" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>1</v>
+      </c>
+      <c r="E33" s="24">
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -4991,37 +4746,71 @@
         <v>40</v>
       </c>
       <c r="D34" s="24">
-        <v>0.26700000000000002</v>
-      </c>
-      <c r="E34" s="24" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
+        <v>0.66749999999999998</v>
+      </c>
+      <c r="E34" s="24">
+        <v>0.66749999999999998</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
-  <conditionalFormatting sqref="A1:XFD1 D2:D19 B3:C4 E3:XFD4 A5 A6:C7 E6:XFD7 A8:XFD12 A13:C15 E13:XFD15 A16:XFD19 A35:XFD1048576 B2:XFD2 F29:XFD34">
-    <cfRule type="expression" dxfId="19" priority="66">
+  <conditionalFormatting sqref="A2:A5">
+    <cfRule type="expression" dxfId="15" priority="39">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B21:C25 C26 B27:C27">
-    <cfRule type="expression" dxfId="18" priority="52">
+  <conditionalFormatting sqref="A20:A34">
+    <cfRule type="expression" dxfId="14" priority="21">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B20:C20 A26:A28 E23 E20">
-    <cfRule type="expression" dxfId="17" priority="53">
+  <conditionalFormatting sqref="A1:XFD1 B3:C4 A6:C7 A13:C15 A35:XFD1048576 F6:XFD19 F2:XFD4 B2:E2 A8:E12 A16:E19">
+    <cfRule type="expression" dxfId="13" priority="83">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B20:C25 C26">
+    <cfRule type="expression" dxfId="12" priority="69">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B27:C28">
+    <cfRule type="expression" dxfId="11" priority="50">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B30:C31">
+    <cfRule type="expression" dxfId="10" priority="30">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B33:C34">
+    <cfRule type="expression" dxfId="9" priority="23">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C29">
+    <cfRule type="expression" dxfId="8" priority="35">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C32">
+    <cfRule type="expression" dxfId="7" priority="28">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:XFD5">
-    <cfRule type="expression" dxfId="16" priority="31">
+    <cfRule type="expression" dxfId="6" priority="48">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D34">
+    <cfRule type="expression" dxfId="5" priority="19">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:D7 D35:E1048576">
-    <cfRule type="dataBar" priority="63">
+    <cfRule type="dataBar" priority="80">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5034,8 +4823,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D8:D10 D5 E3:E4 E6:E7">
-    <cfRule type="dataBar" priority="72">
+  <conditionalFormatting sqref="D8:E10 D5:E5">
+    <cfRule type="dataBar" priority="89">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5048,8 +4837,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D15 D13">
-    <cfRule type="dataBar" priority="61">
+  <conditionalFormatting sqref="D13:E13 D15:E15">
+    <cfRule type="dataBar" priority="78">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5062,8 +4851,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D15">
-    <cfRule type="dataBar" priority="59">
+  <conditionalFormatting sqref="D15:E15">
+    <cfRule type="dataBar" priority="76">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5076,8 +4865,48 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:E2 D2:D19">
-    <cfRule type="dataBar" priority="65">
+  <conditionalFormatting sqref="D20:D34">
+    <cfRule type="dataBar" priority="18">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{7AB2700A-6B81-40CE-9D8E-09F24EE45515}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+    <cfRule type="dataBar" priority="20">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{2A85A53E-8626-4C70-ACB0-05A059847601}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:E1">
+    <cfRule type="dataBar" priority="110">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{0F5F82D7-D9D8-496A-8067-873F84F07A41}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:E19">
+    <cfRule type="dataBar" priority="82">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5091,7 +4920,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11:E12">
-    <cfRule type="dataBar" priority="74">
+    <cfRule type="dataBar" priority="91">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5105,7 +4934,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D16:E17">
-    <cfRule type="dataBar" priority="68">
+    <cfRule type="dataBar" priority="85">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5119,7 +4948,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18:E19">
-    <cfRule type="dataBar" priority="67">
+    <cfRule type="dataBar" priority="84">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5132,8 +4961,18 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D1:E1">
-    <cfRule type="dataBar" priority="93">
+  <conditionalFormatting sqref="F20:XFD34">
+    <cfRule type="expression" dxfId="4" priority="6">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E34">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6:E7">
+    <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5141,273 +4980,12 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0F5F82D7-D9D8-496A-8067-873F84F07A41}</x14:id>
+          <x14:id>{8C6FAC25-AF67-4F2F-9FA2-9DA848FD903A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5">
-    <cfRule type="dataBar" priority="32">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3721D2A3-FECF-4A8D-8467-880D87B6D2BC}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E8:E10">
-    <cfRule type="dataBar" priority="71">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{98CA02A6-D84B-4B8F-8EE0-BCA3C3E37146}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E13:E15">
-    <cfRule type="dataBar" priority="69">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2349AB90-2466-4CCB-9A09-AFC1C523F64F}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E20:E22">
-    <cfRule type="dataBar" priority="58">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{990B53AC-61DA-4898-8173-FDAF9356A9A3}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E21:E22">
-    <cfRule type="expression" dxfId="15" priority="51">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23:E24">
-    <cfRule type="dataBar" priority="57">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E24EC235-1C22-47A2-9E45-98978623B831}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E24:E34">
-    <cfRule type="expression" dxfId="14" priority="28">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E25:E26">
-    <cfRule type="dataBar" priority="50">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{416DB728-3CDE-4A4A-A59B-4A22B9276A40}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E27">
-    <cfRule type="dataBar" priority="56">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{69715B00-4721-4DC7-BD2B-D23473816C64}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E28">
-    <cfRule type="dataBar" priority="48">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A7C290DA-E617-4412-A5C5-3335857A068B}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F20:XFD28 B28:C28">
-    <cfRule type="expression" dxfId="13" priority="33">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A2:A4">
-    <cfRule type="expression" dxfId="12" priority="22">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A29:A31">
-    <cfRule type="expression" dxfId="11" priority="21">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A32:A34">
-    <cfRule type="expression" dxfId="10" priority="20">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C29 B30:C30">
-    <cfRule type="expression" dxfId="9" priority="18">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E29">
-    <cfRule type="dataBar" priority="17">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{300C6859-9C43-4AEC-AFC7-5EFBEDA5FFC9}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E30">
-    <cfRule type="dataBar" priority="19">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4F0D40E6-4588-4F1B-B566-71161E555644}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E31">
-    <cfRule type="dataBar" priority="16">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F85D4A2E-7508-48E4-B231-7EC9DFE30A3A}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B31:C31">
-    <cfRule type="expression" dxfId="8" priority="13">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C32 B33:C33">
-    <cfRule type="expression" dxfId="7" priority="11">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E32">
-    <cfRule type="dataBar" priority="10">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{631841D2-B288-4E38-89D8-A83C71A694E2}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E33">
-    <cfRule type="dataBar" priority="12">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{11D952EA-6F71-484F-992F-FC230678E023}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E34">
-    <cfRule type="dataBar" priority="9">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{66ACFE75-5158-4AB2-B574-39A4A5AFA58F}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B34:C34">
-    <cfRule type="expression" dxfId="6" priority="6">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A20:A22">
-    <cfRule type="expression" dxfId="5" priority="5">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A23:A25">
-    <cfRule type="expression" dxfId="4" priority="4">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D20:D34">
-    <cfRule type="expression" dxfId="3" priority="2">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D20:D34">
+  <conditionalFormatting sqref="E20:E34">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5416,12 +4994,10 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7AB2700A-6B81-40CE-9D8E-09F24EE45515}</x14:id>
+          <x14:id>{7DACECD8-CF17-4DAC-86F1-80FDC5E5A1ED}</x14:id>
         </ext>
       </extLst>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D20:D34">
     <cfRule type="dataBar" priority="3">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5430,12 +5006,12 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A85A53E-8626-4C70-ACB0-05A059847601}</x14:id>
+          <x14:id>{80FA55A8-C539-4A84-98B4-76E995118752}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations xWindow="701" yWindow="283" count="2">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Ratio (1)" prompt="Input/output quantities, relative to process throughput" sqref="D1" xr:uid="{00000000-0002-0000-0400-000000000000}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Ratio at minimum operation point" prompt="Input/Output ratio at point of minimum operation (min-fract in 'Process' sheet)._x000a__x000a_All values have to be larger/equal to ratio!" sqref="E1" xr:uid="{00000000-0002-0000-0400-000001000000}"/>
   </dataValidations>
@@ -5472,7 +5048,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D8:D10 D5 E3:E4 E6:E7</xm:sqref>
+          <xm:sqref>D8:E10 D5:E5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{FD70C683-63D2-4AF7-9844-0053BE6DF679}">
@@ -5487,7 +5063,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D15 D13</xm:sqref>
+          <xm:sqref>D13:E13 D15:E15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{C12684E9-C44A-443A-881A-7ED428CB9718}">
@@ -5502,7 +5078,49 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D15</xm:sqref>
+          <xm:sqref>D15:E15</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{7AB2700A-6B81-40CE-9D8E-09F24EE45515}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <x14:cfRule type="dataBar" id="{2A85A53E-8626-4C70-ACB0-05A059847601}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D20:D34</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{0F5F82D7-D9D8-496A-8067-873F84F07A41}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D1:E1</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{E75D5CC6-8EBE-4E5D-B4DA-5515E5E7F357}">
@@ -5517,7 +5135,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D2:E2 D2:D19</xm:sqref>
+          <xm:sqref>D2:E19</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{F00EA992-7704-4FFF-9390-9F67541314D3}">
@@ -5565,7 +5183,7 @@
           <xm:sqref>D18:E19</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0F5F82D7-D9D8-496A-8067-873F84F07A41}">
+          <x14:cfRule type="dataBar" id="{8C6FAC25-AF67-4F2F-9FA2-9DA848FD903A}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5577,10 +5195,10 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D1:E1</xm:sqref>
+          <xm:sqref>E6:E7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3721D2A3-FECF-4A8D-8467-880D87B6D2BC}">
+          <x14:cfRule type="dataBar" id="{7DACECD8-CF17-4DAC-86F1-80FDC5E5A1ED}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5592,10 +5210,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E5</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{98CA02A6-D84B-4B8F-8EE0-BCA3C3E37146}">
+          <x14:cfRule type="dataBar" id="{80FA55A8-C539-4A84-98B4-76E995118752}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5607,217 +5222,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>E8:E10</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2349AB90-2466-4CCB-9A09-AFC1C523F64F}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E13:E15</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{990B53AC-61DA-4898-8173-FDAF9356A9A3}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E20:E22</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E24EC235-1C22-47A2-9E45-98978623B831}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E23:E24</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{416DB728-3CDE-4A4A-A59B-4A22B9276A40}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E25:E26</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{69715B00-4721-4DC7-BD2B-D23473816C64}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E27</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A7C290DA-E617-4412-A5C5-3335857A068B}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E28</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{300C6859-9C43-4AEC-AFC7-5EFBEDA5FFC9}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E29</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4F0D40E6-4588-4F1B-B566-71161E555644}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E30</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F85D4A2E-7508-48E4-B231-7EC9DFE30A3A}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E31</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{631841D2-B288-4E38-89D8-A83C71A694E2}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E32</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{11D952EA-6F71-484F-992F-FC230678E023}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E33</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{66ACFE75-5158-4AB2-B574-39A4A5AFA58F}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>E34</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7AB2700A-6B81-40CE-9D8E-09F24EE45515}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D20:D34</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2A85A53E-8626-4C70-ACB0-05A059847601}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D20:D34</xm:sqref>
+          <xm:sqref>E20:E34</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -5903,7 +5308,7 @@
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <conditionalFormatting sqref="M1">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6239,12 +5644,12 @@
   <autoFilter ref="A1:U1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="A2:A4">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1">
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Made some adaptions to IR and deltaQ
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA1DD5CA-3F8A-48D5-A956-A4AC9E3200EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867B10B5-66B7-4BCD-B9C8-6C440BFBFF37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -2335,16 +2335,7 @@
     <cellStyle name="Zelle überprüfen 4" xfId="214" xr:uid="{00000000-0005-0000-0000-000092010000}"/>
     <cellStyle name="Zelle überprüfen 5" xfId="215" xr:uid="{00000000-0005-0000-0000-000093010000}"/>
   </cellStyles>
-  <dxfs count="27">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="26">
     <dxf>
       <border>
         <top style="thin">
@@ -3438,10 +3429,10 @@
   <autoFilter ref="B1:F4" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="B1:B1048576">
-    <cfRule type="duplicateValues" dxfId="26" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:B11">
-    <cfRule type="expression" dxfId="25" priority="10">
+    <cfRule type="expression" dxfId="24" priority="10">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4094,47 +4085,47 @@
   <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="A16 A17:XFD1048576">
-    <cfRule type="expression" dxfId="24" priority="41">
+    <cfRule type="expression" dxfId="23" priority="41">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:F13">
-    <cfRule type="expression" dxfId="23" priority="9">
+    <cfRule type="expression" dxfId="22" priority="9">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:XFD1 P2:XFD4 P9:XFD16">
-    <cfRule type="expression" dxfId="22" priority="40">
+    <cfRule type="expression" dxfId="21" priority="40">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G4 G12:G13">
-    <cfRule type="expression" dxfId="21" priority="8">
+    <cfRule type="expression" dxfId="20" priority="8">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H7">
-    <cfRule type="expression" dxfId="20" priority="6">
+    <cfRule type="expression" dxfId="19" priority="6">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:H13">
-    <cfRule type="expression" dxfId="19" priority="1">
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:O2">
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="17" priority="2">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I11:K11">
-    <cfRule type="expression" dxfId="17" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I11:O12">
-    <cfRule type="expression" dxfId="16" priority="3">
+    <cfRule type="expression" dxfId="15" priority="3">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4253,10 +4244,10 @@
         <v>39</v>
       </c>
       <c r="D5" s="24">
-        <v>1.6666666666666667</v>
+        <v>2.04</v>
       </c>
       <c r="E5" s="24">
-        <v>1.6666666666666667</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4287,10 +4278,10 @@
         <v>40</v>
       </c>
       <c r="D7" s="24">
-        <v>0.34166666666666667</v>
+        <v>0.41208</v>
       </c>
       <c r="E7" s="24">
-        <v>0.34166666666666667</v>
+        <v>0.41208</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4755,62 +4746,57 @@
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <conditionalFormatting sqref="A2:A5">
-    <cfRule type="expression" dxfId="15" priority="39">
+    <cfRule type="expression" dxfId="14" priority="40">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A20:A34">
-    <cfRule type="expression" dxfId="14" priority="21">
+    <cfRule type="expression" dxfId="13" priority="22">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:XFD1 B3:C4 A6:C7 A13:C15 A35:XFD1048576 F6:XFD19 F2:XFD4 B2:E2 A8:E12 A16:E19">
-    <cfRule type="expression" dxfId="13" priority="83">
+  <conditionalFormatting sqref="A1:XFD1 B2:E2 F2:XFD4 B3:C4 A6:C7 A8:E12 A13:C15 A16:E19 A35:XFD1048576">
+    <cfRule type="expression" dxfId="12" priority="84">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20:C25 C26">
-    <cfRule type="expression" dxfId="12" priority="69">
+    <cfRule type="expression" dxfId="11" priority="70">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:C28">
-    <cfRule type="expression" dxfId="11" priority="50">
+    <cfRule type="expression" dxfId="10" priority="51">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30:C31">
-    <cfRule type="expression" dxfId="10" priority="30">
+    <cfRule type="expression" dxfId="9" priority="31">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33:C34">
-    <cfRule type="expression" dxfId="9" priority="23">
+    <cfRule type="expression" dxfId="8" priority="24">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C29">
-    <cfRule type="expression" dxfId="8" priority="35">
+    <cfRule type="expression" dxfId="7" priority="36">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C32">
-    <cfRule type="expression" dxfId="7" priority="28">
+    <cfRule type="expression" dxfId="6" priority="29">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:XFD5">
-    <cfRule type="expression" dxfId="6" priority="48">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D34">
-    <cfRule type="expression" dxfId="5" priority="19">
+    <cfRule type="expression" dxfId="5" priority="49">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6:D7 D35:E1048576">
-    <cfRule type="dataBar" priority="80">
+    <cfRule type="dataBar" priority="81">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4823,8 +4809,67 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D20:D34">
+    <cfRule type="dataBar" priority="19">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{7AB2700A-6B81-40CE-9D8E-09F24EE45515}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+    <cfRule type="dataBar" priority="21">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{2A85A53E-8626-4C70-ACB0-05A059847601}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D1:E1">
+    <cfRule type="dataBar" priority="111">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{0F5F82D7-D9D8-496A-8067-873F84F07A41}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:E19">
+    <cfRule type="dataBar" priority="83">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{E75D5CC6-8EBE-4E5D-B4DA-5515E5E7F357}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:E34">
+    <cfRule type="expression" dxfId="4" priority="3">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D8:E10 D5:E5">
-    <cfRule type="dataBar" priority="89">
+    <cfRule type="dataBar" priority="90">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4837,8 +4882,22 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D11:E12">
+    <cfRule type="dataBar" priority="92">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F00EA992-7704-4FFF-9390-9F67541314D3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="D13:E13 D15:E15">
-    <cfRule type="dataBar" priority="78">
+    <cfRule type="dataBar" priority="79">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4852,7 +4911,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15:E15">
-    <cfRule type="dataBar" priority="76">
+    <cfRule type="dataBar" priority="77">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4865,76 +4924,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D20:D34">
-    <cfRule type="dataBar" priority="18">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7AB2700A-6B81-40CE-9D8E-09F24EE45515}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-    <cfRule type="dataBar" priority="20">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2A85A53E-8626-4C70-ACB0-05A059847601}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D1:E1">
-    <cfRule type="dataBar" priority="110">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0F5F82D7-D9D8-496A-8067-873F84F07A41}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:E19">
-    <cfRule type="dataBar" priority="82">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E75D5CC6-8EBE-4E5D-B4DA-5515E5E7F357}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D11:E12">
-    <cfRule type="dataBar" priority="91">
-      <dataBar>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="2"/>
-        <color rgb="FF638EC6"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F00EA992-7704-4FFF-9390-9F67541314D3}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D16:E17">
-    <cfRule type="dataBar" priority="85">
+    <cfRule type="dataBar" priority="86">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4948,7 +4939,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18:E19">
-    <cfRule type="dataBar" priority="84">
+    <cfRule type="dataBar" priority="85">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4961,18 +4952,8 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F20:XFD34">
-    <cfRule type="expression" dxfId="4" priority="6">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E34">
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="E6:E7">
-    <cfRule type="dataBar" priority="4">
+    <cfRule type="dataBar" priority="5">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4986,7 +4967,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E20:E34">
-    <cfRule type="dataBar" priority="1">
+    <cfRule type="dataBar" priority="2">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -4998,7 +4979,7 @@
         </ext>
       </extLst>
     </cfRule>
-    <cfRule type="dataBar" priority="3">
+    <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="2"/>
@@ -5007,6 +4988,25 @@
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{80FA55A8-C539-4A84-98B4-76E995118752}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F6:XFD34">
+    <cfRule type="expression" dxfId="3" priority="7">
+      <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="2"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F74817C3-D28A-45F6-A051-86E1B85965F4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5034,51 +5034,6 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>D6:D7 D35:E1048576</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4EFF1923-5632-46D2-BEE4-19792B834F3E}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D8:E10 D5:E5</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FD70C683-63D2-4AF7-9844-0053BE6DF679}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D13:E13 D15:E15</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C12684E9-C44A-443A-881A-7ED428CB9718}">
-            <x14:dataBar minLength="0" maxLength="100" gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>2</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D15:E15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{7AB2700A-6B81-40CE-9D8E-09F24EE45515}">
@@ -5138,6 +5093,21 @@
           <xm:sqref>D2:E19</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{4EFF1923-5632-46D2-BEE4-19792B834F3E}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D8:E10 D5:E5</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{F00EA992-7704-4FFF-9390-9F67541314D3}">
             <x14:dataBar minLength="0" maxLength="100" gradient="0">
               <x14:cfvo type="num">
@@ -5151,6 +5121,36 @@
             </x14:dataBar>
           </x14:cfRule>
           <xm:sqref>D11:E12</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{FD70C683-63D2-4AF7-9844-0053BE6DF679}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D13:E13 D15:E15</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{C12684E9-C44A-443A-881A-7ED428CB9718}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D15:E15</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{04E5CAC7-3551-4B94-B47C-699E9D4FD15E}">
@@ -5224,6 +5224,21 @@
           </x14:cfRule>
           <xm:sqref>E20:E34</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F74817C3-D28A-45F6-A051-86E1B85965F4}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>2</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>E7</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>
@@ -5308,7 +5323,7 @@
   </sheetData>
   <autoFilter ref="A1:N1" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <conditionalFormatting sqref="M1">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5644,12 +5659,12 @@
   <autoFilter ref="A1:U1" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <conditionalFormatting sqref="A2:A4">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="1" priority="1">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S1">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>NOT(EXACT(INDIRECT("Z"&amp;ROW()-1&amp;"S1",FALSE()), INDIRECT("Z"&amp;ROW()&amp;"S1",FALSE())))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
running with wacc again at 0.071
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D83EA04-9730-41E6-B4A7-C16CB7838C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75BC9D8-1D2B-4522-99B7-8C15BF492660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-5565" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -2866,12 +2866,12 @@
     <tabColor rgb="FFC00000"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.109375" style="31" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" style="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="74.88671875" style="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="11.44140625" style="31"/>
+    <col min="1" max="1" width="14.140625" style="31" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" style="31" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="74.85546875" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.42578125" style="31"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2907,7 +2907,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="43.2">
+    <row r="4" spans="1:3" ht="45">
       <c r="A4" s="32" t="s">
         <v>60</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="28.8">
+    <row r="6" spans="1:3" ht="30">
       <c r="A6" s="32" t="s">
         <v>71</v>
       </c>
@@ -2958,9 +2958,9 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" width="11.44140625" style="1"/>
+    <col min="1" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="14" customFormat="1">
@@ -3088,9 +3088,9 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="16384" width="11.44140625" style="1"/>
+    <col min="1" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="14" customFormat="1">
@@ -3116,9 +3116,9 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" style="1"/>
+    <col min="1" max="1" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3206,9 +3206,9 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3242,15 +3242,15 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="8" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="13.88671875" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.44140625" style="2"/>
+    <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="8" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customFormat="1">
@@ -3506,22 +3506,22 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:O13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="10.6640625" style="19" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" style="19" customWidth="1"/>
-    <col min="7" max="7" width="18.109375" style="19" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="10.7109375" style="19" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" style="19" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="2" customWidth="1"/>
     <col min="9" max="9" width="24" style="19" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" customWidth="1"/>
-    <col min="11" max="11" width="10.6640625" style="21" customWidth="1"/>
-    <col min="12" max="12" width="16.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5546875" style="2" customWidth="1"/>
-    <col min="14" max="14" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="11.44140625" style="2"/>
+    <col min="10" max="10" width="10.7109375" style="19" customWidth="1"/>
+    <col min="11" max="11" width="10.7109375" style="21" customWidth="1"/>
+    <col min="12" max="12" width="16.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" style="2" customWidth="1"/>
+    <col min="14" max="14" width="14.85546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" customFormat="1">
@@ -3923,7 +3923,7 @@
         <v>27</v>
       </c>
       <c r="H9" s="2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I9" s="52">
         <v>1951271.6999999997</v>
@@ -3970,7 +3970,7 @@
         <v>27</v>
       </c>
       <c r="H10" s="2">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="I10" s="51">
         <v>5909565.7200000007</v>
@@ -4111,7 +4111,7 @@
         <v>27</v>
       </c>
       <c r="H13" s="2">
-        <v>0.44</v>
+        <v>0</v>
       </c>
       <c r="I13" s="55">
         <v>5648000</v>
@@ -4209,14 +4209,14 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:E34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.44140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="20" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" style="20" customWidth="1"/>
-    <col min="6" max="16384" width="11.44140625" style="2"/>
+    <col min="1" max="1" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="20" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" style="20" customWidth="1"/>
+    <col min="6" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" customFormat="1">
@@ -5305,20 +5305,20 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="10.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.6640625" style="20" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" style="19" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" style="22" customWidth="1"/>
-    <col min="10" max="13" width="10.6640625" style="19" customWidth="1"/>
-    <col min="14" max="14" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.7109375" style="20" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" style="19" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" style="22" customWidth="1"/>
+    <col min="10" max="13" width="10.7109375" style="19" customWidth="1"/>
+    <col min="14" max="14" width="14.85546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -5406,28 +5406,28 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:W4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.88671875" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.6640625" style="22" customWidth="1"/>
-    <col min="12" max="12" width="12.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.7109375" style="22" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.140625" style="22" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" style="19" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.6640625" style="22" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.44140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="17" max="19" width="12.109375" style="22" customWidth="1"/>
-    <col min="20" max="20" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.6640625" style="22" customWidth="1"/>
-    <col min="22" max="22" width="12.109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.44140625" style="2"/>
+    <col min="15" max="15" width="11.7109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.42578125" style="22" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="12.140625" style="22" customWidth="1"/>
+    <col min="20" max="20" width="14.85546875" style="22" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.7109375" style="22" customWidth="1"/>
+    <col min="22" max="22" width="12.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.42578125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -5755,13 +5755,13 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.33203125" style="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5830,11 +5830,11 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" style="1"/>
-    <col min="2" max="2" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.44140625" style="1"/>
+    <col min="1" max="1" width="11.42578125" style="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
coal phase out by 2030 according to 1.5 degree target
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75BC9D8-1D2B-4522-99B7-8C15BF492660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A190835-8D4D-42A6-AFF5-258C33D2A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" tabRatio="796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -2866,12 +2866,12 @@
     <tabColor rgb="FFC00000"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.140625" style="31" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" style="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="74.85546875" style="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="11.42578125" style="31"/>
+    <col min="1" max="1" width="14.109375" style="31" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" style="31" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="74.88671875" style="31" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.44140625" style="31"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2907,7 +2907,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="45">
+    <row r="4" spans="1:3" ht="43.2">
       <c r="A4" s="32" t="s">
         <v>60</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="30">
+    <row r="6" spans="1:3" ht="28.8">
       <c r="A6" s="32" t="s">
         <v>71</v>
       </c>
@@ -2958,9 +2958,9 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="14" customFormat="1">
@@ -3088,9 +3088,9 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="14" customFormat="1">
@@ -3116,9 +3116,9 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3206,9 +3206,9 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3242,15 +3242,15 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="8" customWidth="1"/>
-    <col min="5" max="5" width="16.28515625" style="8" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="13.88671875" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" customFormat="1">
@@ -3506,22 +3506,22 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:O13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="10.7109375" style="19" customWidth="1"/>
-    <col min="6" max="6" width="20.140625" style="19" customWidth="1"/>
-    <col min="7" max="7" width="18.140625" style="19" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="10.6640625" style="19" customWidth="1"/>
+    <col min="6" max="6" width="20.109375" style="19" customWidth="1"/>
+    <col min="7" max="7" width="18.109375" style="19" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="2" customWidth="1"/>
     <col min="9" max="9" width="24" style="19" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="19" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" style="21" customWidth="1"/>
-    <col min="12" max="12" width="16.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" style="2" customWidth="1"/>
-    <col min="14" max="14" width="14.85546875" style="22" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="11.42578125" style="2"/>
+    <col min="10" max="10" width="10.6640625" style="19" customWidth="1"/>
+    <col min="11" max="11" width="10.6640625" style="21" customWidth="1"/>
+    <col min="12" max="12" width="16.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5546875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" customFormat="1">
@@ -3582,7 +3582,7 @@
         <v>56122</v>
       </c>
       <c r="D2" s="19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="19">
         <v>0</v>
@@ -3629,7 +3629,7 @@
         <v>43599</v>
       </c>
       <c r="D3" s="19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="19">
         <v>0</v>
@@ -4209,14 +4209,14 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:E34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" style="20" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" style="20" customWidth="1"/>
-    <col min="6" max="16384" width="11.42578125" style="2"/>
+    <col min="1" max="1" width="16.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="18.5546875" style="20" customWidth="1"/>
+    <col min="6" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" customFormat="1">
@@ -5305,20 +5305,20 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="2" width="10.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.7109375" style="20" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" style="19" customWidth="1"/>
-    <col min="9" max="9" width="10.7109375" style="22" customWidth="1"/>
-    <col min="10" max="13" width="10.7109375" style="19" customWidth="1"/>
-    <col min="14" max="14" width="14.85546875" style="22" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.6640625" style="20" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="19" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="22" customWidth="1"/>
+    <col min="10" max="13" width="10.6640625" style="19" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -5406,28 +5406,28 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:W4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" style="19" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.85546875" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.7109375" style="22" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" style="19" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="10.6640625" style="22" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" style="22" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12" style="19" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.7109375" style="22" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.42578125" style="22" bestFit="1" customWidth="1"/>
-    <col min="17" max="19" width="12.140625" style="22" customWidth="1"/>
-    <col min="20" max="20" width="14.85546875" style="22" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.7109375" style="22" customWidth="1"/>
-    <col min="22" max="22" width="12.140625" style="22" bestFit="1" customWidth="1"/>
-    <col min="23" max="16384" width="11.42578125" style="2"/>
+    <col min="15" max="15" width="11.6640625" style="22" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.44140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="17" max="19" width="12.109375" style="22" customWidth="1"/>
+    <col min="20" max="20" width="14.88671875" style="22" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" style="22" customWidth="1"/>
+    <col min="22" max="22" width="12.109375" style="22" bestFit="1" customWidth="1"/>
+    <col min="23" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -5755,13 +5755,13 @@
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.28515625" style="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.33203125" style="34" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -5830,11 +5830,11 @@
     <tabColor theme="9" tint="0.39997558519241921"/>
   </sheetPr>
   <dimension ref="A1:B14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" style="1"/>
-    <col min="2" max="2" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.42578125" style="1"/>
+    <col min="1" max="1" width="11.44140625" style="1"/>
+    <col min="2" max="2" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">

</xml_diff>

<commit_message>
Added a lot of new Plotting features
</commit_message>
<xml_diff>
--- a/Input/urbs_intertemporal_2050/2024.xlsx
+++ b/Input/urbs_intertemporal_2050/2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\Input\urbs_intertemporal_2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A190835-8D4D-42A6-AFF5-258C33D2A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC16133-A31F-4DE5-ABF4-ED064CE0553F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="796" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global" sheetId="11" r:id="rId1"/>
@@ -3241,7 +3241,7 @@
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="2" customWidth="1"/>
@@ -3253,7 +3253,7 @@
     <col min="7" max="16384" width="11.44140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" customFormat="1">
+    <row r="1" spans="1:14" customFormat="1">
       <c r="A1" t="s">
         <v>43</v>
       </c>
@@ -3273,7 +3273,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:14">
       <c r="A2" s="3" t="s">
         <v>93</v>
       </c>
@@ -3296,7 +3296,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:14">
       <c r="A3" s="3" t="s">
         <v>93</v>
       </c>
@@ -3319,7 +3319,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:14">
       <c r="A4" s="3" t="s">
         <v>93</v>
       </c>
@@ -3338,8 +3338,13 @@
       <c r="F4" s="7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4"/>
+      <c r="N4"/>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="3" t="s">
         <v>93</v>
       </c>
@@ -3358,8 +3363,13 @@
       <c r="F5" s="7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="J5"/>
+      <c r="K5"/>
+      <c r="L5"/>
+      <c r="M5"/>
+      <c r="N5"/>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" s="3" t="s">
         <v>93</v>
       </c>
@@ -3378,8 +3388,13 @@
       <c r="F6" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="J6"/>
+      <c r="K6"/>
+      <c r="L6"/>
+      <c r="M6"/>
+      <c r="N6"/>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" s="3" t="s">
         <v>93</v>
       </c>
@@ -3398,8 +3413,13 @@
       <c r="F7" s="7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7"/>
+      <c r="N7"/>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" s="3" t="s">
         <v>93</v>
       </c>
@@ -3419,7 +3439,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:14">
       <c r="A9" s="3" t="s">
         <v>93</v>
       </c>
@@ -3439,7 +3459,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:14">
       <c r="A10" s="3" t="s">
         <v>93</v>
       </c>
@@ -3459,7 +3479,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:14">
       <c r="A11" s="3" t="s">
         <v>93</v>
       </c>

</xml_diff>